<commit_message>
version 35 - Implement Payment and Shopping bag with combined database
</commit_message>
<xml_diff>
--- a/API_Documentation/RESTFul_API.xlsx
+++ b/API_Documentation/RESTFul_API.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Server APIs" sheetId="3" r:id="rId1"/>
@@ -661,12 +661,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <charset val="134"/>
-      </rPr>
       <t>+ If user is valid:</t>
     </r>
     <r>
@@ -883,8 +877,27 @@
     <t>/api/payment_handling</t>
   </si>
   <si>
-    <t>- Check request header to get current user and persional shopping bag 
-in session storage</t>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">- Check request header to get current user and persional shopping bag 
+in Redis or DB </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(only applicable for Scenario 2: If want user must login before access the website)</t>
+    </r>
   </si>
   <si>
     <t>[{
@@ -999,7 +1012,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="33">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1215,6 +1228,14 @@
     </font>
     <font>
       <b/>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
@@ -1225,7 +1246,7 @@
       <charset val="0"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="41">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1265,6 +1286,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.25"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1643,7 +1670,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1667,16 +1694,16 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1685,89 +1712,89 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1881,34 +1908,28 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1939,7 +1960,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1950,7 +1971,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
@@ -2326,11 +2347,11 @@
       </c>
       <c r="I2" s="12"/>
       <c r="J2" s="12"/>
-      <c r="K2" s="47" t="s">
+      <c r="K2" s="45" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" ht="35.4" customHeight="1" spans="1:11">
+    <row r="3" s="1" customFormat="1" ht="23" customHeight="1" spans="1:11">
       <c r="A3" s="6"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -2353,7 +2374,7 @@
       <c r="J3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="48"/>
+      <c r="K3" s="46"/>
     </row>
     <row r="4" s="2" customFormat="1" ht="54" customHeight="1" spans="1:11">
       <c r="A4" s="15" t="s">
@@ -2368,13 +2389,13 @@
       <c r="D4" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="52" t="s">
+      <c r="E4" s="50" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="52" t="s">
+      <c r="G4" s="50" t="s">
         <v>18</v>
       </c>
       <c r="H4" s="20" t="s">
@@ -2382,7 +2403,7 @@
       </c>
       <c r="I4" s="25"/>
       <c r="J4" s="25"/>
-      <c r="K4" s="53" t="s">
+      <c r="K4" s="51" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2399,13 +2420,13 @@
       <c r="D5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="52" t="s">
+      <c r="E5" s="50" t="s">
         <v>24</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="52" t="s">
+      <c r="G5" s="50" t="s">
         <v>25</v>
       </c>
       <c r="H5" s="20" t="s">
@@ -2413,7 +2434,7 @@
       </c>
       <c r="I5" s="25"/>
       <c r="J5" s="25"/>
-      <c r="K5" s="49" t="s">
+      <c r="K5" s="47" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2429,16 +2450,16 @@
       </c>
       <c r="F6" s="25"/>
       <c r="G6" s="25"/>
-      <c r="H6" s="52" t="s">
+      <c r="H6" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="52" t="s">
+      <c r="I6" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="52" t="s">
+      <c r="J6" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="49" t="s">
+      <c r="K6" s="47" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2449,7 +2470,7 @@
       <c r="D7" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="52" t="s">
         <v>33</v>
       </c>
       <c r="F7" s="26"/>
@@ -2459,7 +2480,7 @@
       </c>
       <c r="I7" s="25"/>
       <c r="J7" s="25"/>
-      <c r="K7" s="49" t="s">
+      <c r="K7" s="47" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2475,7 +2496,7 @@
       </c>
       <c r="F8" s="25"/>
       <c r="G8" s="25"/>
-      <c r="H8" s="55" t="s">
+      <c r="H8" s="53" t="s">
         <v>36</v>
       </c>
       <c r="I8" s="27" t="s">
@@ -2498,7 +2519,7 @@
       <c r="E9" s="20"/>
       <c r="F9" s="25"/>
       <c r="G9" s="25"/>
-      <c r="H9" s="55" t="s">
+      <c r="H9" s="53" t="s">
         <v>41</v>
       </c>
       <c r="I9" s="27" t="s">
@@ -2777,7 +2798,7 @@
       </c>
       <c r="I19" s="25"/>
       <c r="J19" s="25"/>
-      <c r="K19" s="50" t="s">
+      <c r="K19" s="48" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2798,7 +2819,7 @@
       </c>
       <c r="I20" s="25"/>
       <c r="J20" s="25"/>
-      <c r="K20" s="51" t="s">
+      <c r="K20" s="49" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2819,7 +2840,7 @@
       </c>
       <c r="I21" s="25"/>
       <c r="J21" s="25"/>
-      <c r="K21" s="51" t="s">
+      <c r="K21" s="49" t="s">
         <v>91</v>
       </c>
     </row>
@@ -2840,7 +2861,7 @@
       </c>
       <c r="I22" s="25"/>
       <c r="J22" s="25"/>
-      <c r="K22" s="51" t="s">
+      <c r="K22" s="49" t="s">
         <v>93</v>
       </c>
     </row>
@@ -2857,13 +2878,13 @@
       <c r="D23" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="E23" s="52" t="s">
+      <c r="E23" s="50" t="s">
         <v>98</v>
       </c>
-      <c r="F23" s="52" t="s">
+      <c r="F23" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="G23" s="52" t="s">
+      <c r="G23" s="50" t="s">
         <v>100</v>
       </c>
       <c r="H23" s="20" t="s">
@@ -2871,7 +2892,7 @@
       </c>
       <c r="I23" s="25"/>
       <c r="J23" s="25"/>
-      <c r="K23" s="56" t="s">
+      <c r="K23" s="54" t="s">
         <v>102</v>
       </c>
     </row>
@@ -2887,7 +2908,7 @@
       </c>
       <c r="F24" s="25"/>
       <c r="G24" s="25"/>
-      <c r="H24" s="52" t="s">
+      <c r="H24" s="50" t="s">
         <v>104</v>
       </c>
       <c r="I24" s="19" t="s">
@@ -2896,7 +2917,7 @@
       <c r="J24" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="K24" s="49" t="s">
+      <c r="K24" s="47" t="s">
         <v>107</v>
       </c>
     </row>
@@ -2918,16 +2939,16 @@
       </c>
       <c r="F25" s="25"/>
       <c r="G25" s="25"/>
-      <c r="H25" s="52" t="s">
+      <c r="H25" s="50" t="s">
         <v>112</v>
       </c>
       <c r="I25" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="J25" s="57" t="s">
+      <c r="J25" s="55" t="s">
         <v>114</v>
       </c>
-      <c r="K25" s="49" t="s">
+      <c r="K25" s="47" t="s">
         <v>115</v>
       </c>
     </row>
@@ -2943,16 +2964,16 @@
       </c>
       <c r="F26" s="25"/>
       <c r="G26" s="25"/>
-      <c r="H26" s="52" t="s">
+      <c r="H26" s="50" t="s">
         <v>117</v>
       </c>
       <c r="I26" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="J26" s="57" t="s">
+      <c r="J26" s="55" t="s">
         <v>119</v>
       </c>
-      <c r="K26" s="49" t="s">
+      <c r="K26" s="47" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2969,13 +2990,13 @@
       <c r="D27" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="58" t="s">
+      <c r="E27" s="56" t="s">
         <v>124</v>
       </c>
       <c r="F27" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G27" s="57" t="s">
+      <c r="G27" s="55" t="s">
         <v>125</v>
       </c>
       <c r="H27" s="20" t="s">
@@ -3010,7 +3031,7 @@
       </c>
       <c r="I28" s="25"/>
       <c r="J28" s="25"/>
-      <c r="K28" s="53" t="s">
+      <c r="K28" s="51" t="s">
         <v>131</v>
       </c>
     </row>
@@ -3018,22 +3039,22 @@
       <c r="A29" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="B29" s="39" t="s">
+      <c r="B29" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="C29" s="39" t="s">
+      <c r="C29" s="22" t="s">
         <v>134</v>
       </c>
       <c r="D29" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="59" t="s">
+      <c r="E29" s="57" t="s">
         <v>135</v>
       </c>
-      <c r="F29" s="19" t="s">
+      <c r="F29" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="G29" s="19" t="s">
+      <c r="G29" s="40" t="s">
         <v>136</v>
       </c>
       <c r="H29" s="20" t="s">
@@ -3041,14 +3062,14 @@
       </c>
       <c r="I29" s="25"/>
       <c r="J29" s="25"/>
-      <c r="K29" s="49" t="s">
+      <c r="K29" s="47" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="30" ht="258.6" customHeight="1" spans="1:11">
       <c r="A30" s="41"/>
-      <c r="B30" s="42"/>
-      <c r="C30" s="42"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
       <c r="D30" s="18" t="s">
         <v>138</v>
       </c>
@@ -3057,30 +3078,30 @@
       </c>
       <c r="F30" s="25"/>
       <c r="G30" s="25"/>
-      <c r="H30" s="52" t="s">
+      <c r="H30" s="50" t="s">
         <v>139</v>
       </c>
       <c r="I30" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="J30" s="52" t="s">
+      <c r="J30" s="50" t="s">
         <v>141</v>
       </c>
-      <c r="K30" s="49" t="s">
+      <c r="K30" s="47" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="31" ht="141" customHeight="1" spans="1:11">
-      <c r="A31" s="43"/>
-      <c r="B31" s="44"/>
-      <c r="C31" s="44"/>
+      <c r="A31" s="42"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
       <c r="D31" s="18" t="s">
         <v>143</v>
       </c>
       <c r="E31" s="20"/>
       <c r="F31" s="25"/>
       <c r="G31" s="25"/>
-      <c r="H31" s="52" t="s">
+      <c r="H31" s="50" t="s">
         <v>144</v>
       </c>
       <c r="I31" s="19" t="s">
@@ -3089,7 +3110,7 @@
       <c r="J31" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="K31" s="49" t="s">
+      <c r="K31" s="47" t="s">
         <v>146</v>
       </c>
     </row>
@@ -3133,13 +3154,13 @@
       <c r="D33" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="E33" s="45" t="s">
+      <c r="E33" s="43" t="s">
         <v>156</v>
       </c>
-      <c r="F33" s="46" t="s">
+      <c r="F33" s="44" t="s">
         <v>157</v>
       </c>
-      <c r="G33" s="46" t="s">
+      <c r="G33" s="44" t="s">
         <v>158</v>
       </c>
       <c r="H33" s="20" t="s">

</xml_diff>